<commit_message>
commit update tabeau de synthese
</commit_message>
<xml_diff>
--- a/dist/docs/TABLEAU_SYNTHESE_E5_2026.xlsx
+++ b/dist/docs/TABLEAU_SYNTHESE_E5_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Baron\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eurof\Documents\Epreuve E5- Portfolio\Tableau de synthese\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ACB0D0A-7D49-47BC-9B6B-413C544A4DF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C3020A-B225-471B-93AC-6ECFA7BE0F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="57">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -101,18 +101,12 @@
 (intitulé et liste des documents et productions associés)</t>
   </si>
   <si>
-    <t xml:space="preserve">N° candidat : </t>
-  </si>
-  <si>
     <t>Réalisations en milieu professionnel en cours de première année</t>
   </si>
   <si>
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
-    <t>Adresse URL du portfolio :</t>
-  </si>
-  <si>
     <t>SESSION 2026</t>
   </si>
   <si>
@@ -143,9 +137,6 @@
     <t>Atelier GSB Gestion des frais en php</t>
   </si>
   <si>
-    <t>Atelier GSB Medicinal Android</t>
-  </si>
-  <si>
     <t>Veille technologique: Données Biométriques (empreintes digitales)</t>
   </si>
   <si>
@@ -213,6 +204,15 @@
   </si>
   <si>
     <t>Période (sous la forme du 26/09/2024 au 30/06/2026)</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://hannabar.github.io/portfolio-hannabar</t>
+  </si>
+  <si>
+    <t>N° candidat : 2544756720</t>
+  </si>
+  <si>
+    <t>Atelier GSB Medicine App Android</t>
   </si>
 </sst>
 </file>
@@ -751,6 +751,18 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -769,6 +781,15 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -816,27 +837,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1220,66 +1220,66 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AQ73"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.90625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="29.77734375" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.44140625" customWidth="1"/>
-    <col min="44" max="16384" width="10.88671875" style="1"/>
+    <col min="1" max="1" width="70.453125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="29.81640625" style="1" customWidth="1"/>
+    <col min="3" max="8" width="18.6328125" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.453125" customWidth="1"/>
+    <col min="44" max="16384" width="10.90625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="H1" s="23"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="27"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="35" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="41" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="36"/>
-      <c r="H3" s="42"/>
+      <c r="A3" s="42" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="48" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="43"/>
+      <c r="H3" s="49"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="38" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="40"/>
+      <c r="A4" s="45" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
       <c r="F4" s="13" t="s">
         <v>8</v>
       </c>
@@ -1291,23 +1291,23 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="34"/>
+      <c r="A5" s="39" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="40"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="41"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="30" t="s">
-        <v>56</v>
+      <c r="B6" s="37" t="s">
+        <v>53</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>0</v>
@@ -1329,9 +1329,9 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="22"/>
-      <c r="B7" s="31"/>
-      <c r="C7" s="47" t="s">
+      <c r="A7" s="26"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="22" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="8" t="s">
@@ -1385,17 +1385,17 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="24" t="s">
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
+      <c r="A8" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1434,22 +1434,20 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="16"/>
-      <c r="F9" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" s="16"/>
+        <v>37</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="H9" s="17"/>
       <c r="I9"/>
       <c r="J9"/>
@@ -1489,22 +1487,20 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="46" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="16"/>
-      <c r="F10" s="48" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="16"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="23"/>
+      <c r="G10" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="H10" s="17"/>
       <c r="I10"/>
       <c r="J10"/>
@@ -1542,25 +1538,19 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="46" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>27</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="15"/>
       <c r="D11" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="48" t="s">
-        <v>27</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E11" s="15"/>
+      <c r="F11" s="23"/>
       <c r="G11" s="16"/>
       <c r="H11" s="17"/>
       <c r="I11"/>
@@ -1599,25 +1589,19 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>27</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="15"/>
       <c r="D12" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="15" t="s">
-        <v>27</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
       <c r="G12" s="16"/>
       <c r="H12" s="17"/>
       <c r="I12"/>
@@ -1656,25 +1640,19 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="46" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="15" t="s">
         <v>27</v>
       </c>
+      <c r="B13" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="15"/>
       <c r="D13" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>27</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
       <c r="G13" s="16"/>
       <c r="H13" s="17"/>
       <c r="I13"/>
@@ -1713,18 +1691,16 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="46" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>27</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="15"/>
       <c r="D14" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
@@ -1766,18 +1742,16 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B15" s="46" t="s">
-        <v>54</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>27</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="15"/>
       <c r="D15" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
@@ -1819,22 +1793,22 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B16" s="46" t="s">
-        <v>47</v>
+        <v>29</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>44</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E16" s="16"/>
       <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
+      <c r="G16" s="15"/>
       <c r="H16" s="17"/>
       <c r="I16"/>
       <c r="J16"/>
@@ -1872,27 +1846,27 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="46" t="s">
-        <v>48</v>
+        <v>30</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>45</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="G17" s="48" t="s">
-        <v>27</v>
+        <v>25</v>
+      </c>
+      <c r="G17" s="23" t="s">
+        <v>25</v>
       </c>
       <c r="H17" s="17"/>
       <c r="I17"/>
@@ -1931,27 +1905,25 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B18" s="46" t="s">
-        <v>49</v>
+        <v>56</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>46</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>27</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E18" s="15"/>
       <c r="F18" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H18" s="17"/>
       <c r="I18"/>
@@ -1990,22 +1962,22 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B19" s="46" t="s">
-        <v>50</v>
+        <v>32</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>47</v>
       </c>
       <c r="C19" s="15"/>
       <c r="D19" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
-      <c r="H19" s="49" t="s">
-        <v>27</v>
+      <c r="H19" s="24" t="s">
+        <v>25</v>
       </c>
       <c r="I19"/>
       <c r="J19"/>
@@ -2043,22 +2015,22 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B20" s="46" t="s">
-        <v>50</v>
+        <v>31</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>47</v>
       </c>
       <c r="C20" s="15"/>
       <c r="D20" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
       <c r="G20" s="16"/>
-      <c r="H20" s="49" t="s">
-        <v>27</v>
+      <c r="H20" s="24" t="s">
+        <v>25</v>
       </c>
       <c r="I20"/>
       <c r="J20"/>
@@ -2096,28 +2068,26 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="B21" s="46" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>27</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="15"/>
       <c r="D21" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G21" s="16"/>
-      <c r="H21" s="49" t="s">
-        <v>27</v>
+      <c r="H21" s="24" t="s">
+        <v>25</v>
       </c>
       <c r="I21"/>
       <c r="J21"/>
@@ -2155,17 +2125,17 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="44"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="44"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="45"/>
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="32"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="33"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -2204,25 +2174,25 @@
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B23" s="46" t="s">
-        <v>52</v>
+        <v>34</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>49</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="G23" s="16"/>
-      <c r="H23" s="49" t="s">
-        <v>27</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H23" s="24"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -2259,17 +2229,17 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A24" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="28"/>
-      <c r="C24" s="28"/>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28"/>
-      <c r="H24" s="29"/>
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
+      <c r="A24" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="35"/>
+      <c r="G24" s="35"/>
+      <c r="H24" s="36"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -2308,25 +2278,25 @@
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="B25" s="46" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="D25" s="16"/>
-      <c r="E25" s="15" t="s">
-        <v>27</v>
-      </c>
+      <c r="D25" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="15"/>
       <c r="F25" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="G25" s="16"/>
-      <c r="H25" s="49" t="s">
-        <v>27</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="G25" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H25" s="24"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2408,7 +2378,7 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.25">
       <c r="A27" s="5"/>
       <c r="B27" s="3"/>
       <c r="C27" s="4"/>

</xml_diff>